<commit_message>
docs(huong-dan): update the Excel import guide for the 0.2.77 templates
The purchase sheet takes one row per finished-goods grade and the stock sheet
treats signed contracts as records with a start and a delivery date. Bundled
sample workbooks re-downloaded from the current templates (they were three
versions behind and also missed the contract code column on the sales sheet).
</commit_message>
<xml_diff>
--- a/docs/huong-dan/nhap-lieu-bang-excel/mau/mau-thu-mua.xlsx
+++ b/docs/huong-dan/nhap-lieu-bang-excel/mau/mau-thu-mua.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -472,9 +472,10 @@
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -487,7 +488,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mỗi dòng = 1 đơn vị / 1 ngày. Đơn giá ghi vào kho 'Giá mủ nguyên liệu'. Mủ nước luôn theo độ TSC; mủ chén theo cột 'Đơn giá mủ chén tính theo'.</t>
+          <t>Mủ nước / mủ chén: mỗi đơn vị 1 dòng / 1 ngày. Đơn giá ghi vào kho 'Giá mủ nguyên liệu'. Mủ nước luôn theo độ TSC; mủ chén theo cột 'Đơn giá mủ chén tính theo'. THU MUA THÀNH PHẨM tính theo CHỦNG LOẠI: mua mấy chủng loại thì thêm bấy nhiêu dòng cho cùng (đơn vị, ngày) — các cột mủ nước/mủ chén chỉ điền ở dòng đầu, dòng sau để trống. File có dòng thành phẩm sẽ GHI ĐÈ toàn bộ phần thành phẩm của ngày đó; không có dòng nào thì phần thành phẩm đã nhập trên web được giữ nguyên.</t>
         </is>
       </c>
     </row>
@@ -536,17 +537,22 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
+          <t>Chủng loại thành phẩm</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
           <t>SL thu mua thành phẩm</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Đơn giá thành phẩm (VNĐ)</t>
-        </is>
-      </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Đơn giá thành phẩm (ngoại tệ)</t>
+          <t>Đơn giá thành phẩm</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Đơn giá thành phẩm bằng</t>
         </is>
       </c>
     </row>
@@ -584,28 +590,39 @@
       </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
+          <t>chỉ dòng thu mua thành phẩm</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
           <t>tấn</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>triệu đ/tấn</t>
-        </is>
-      </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>USD/tấn</t>
+          <t>triệu đ/tấn khi VND · USD/tấn khi USD</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>VND | USD</t>
         </is>
       </c>
     </row>
     <row r="7"/>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="4">
     <dataValidation sqref="A7:A506" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='Danh mục'!$A$2:$A$40</formula1>
     </dataValidation>
     <dataValidation sqref="G7:G506" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Độ TSC,Độ DRC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H7:H506" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SVR CV 50,SVR CV60,SVR L,SVR 3L Mix,SVR 3L,SVR 5S,SVR 5,SVR 10 Mix,SVR 10 / CSR 10,SVR 20 / CSR 20,RSS 3,RSS 1,LATEX,Skim Block,SVR 10CV / 20CV,Chủng loại khác"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K7:K506" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"VND,USD"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>